<commit_message>
Implement Gemini SSE Chat Backend with LangChain integration and initial provider comparison
</commit_message>
<xml_diff>
--- a/comparision.xlsx
+++ b/comparision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AI_Engineering\AI_Engineering\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43869239-B5F3-459E-B352-A23AA1B5ECD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76BD056C-F25B-4A09-A8DA-33A2D077F4B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="22">
   <si>
     <t>gemini-3.5-flash</t>
   </si>
@@ -58,6 +58,42 @@
   </si>
   <si>
     <t>Explain what is API in short.</t>
+  </si>
+  <si>
+    <t>Explain what an API is to a junior software developer in exactly 3 paragraphs. Include one practical example.</t>
+  </si>
+  <si>
+    <t>groq</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>1.64s</t>
+  </si>
+  <si>
+    <t>2.25s</t>
+  </si>
+  <si>
+    <t>1.86s</t>
+  </si>
+  <si>
+    <t>STOP</t>
+  </si>
+  <si>
+    <t>gemini</t>
+  </si>
+  <si>
+    <t>stop</t>
+  </si>
+  <si>
+    <t>17.83s</t>
+  </si>
+  <si>
+    <t>6.10s</t>
+  </si>
+  <si>
+    <t>10.19s</t>
   </si>
 </sst>
 </file>
@@ -99,10 +135,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -384,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:G6"/>
+  <dimension ref="A2:H17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.6640625" bestFit="1" customWidth="1"/>
@@ -396,7 +435,7 @@
     <col min="7" max="7" width="16.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -418,8 +457,11 @@
       <c r="G2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -442,7 +484,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C4">
         <v>8</v>
       </c>
@@ -456,7 +498,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C5">
         <v>8</v>
       </c>
@@ -470,7 +512,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C6">
         <v>8</v>
       </c>
@@ -484,7 +526,174 @@
         <v>623</v>
       </c>
     </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>2</v>
+      </c>
+      <c r="F10" t="s">
+        <v>3</v>
+      </c>
+      <c r="G10" t="s">
+        <v>4</v>
+      </c>
+      <c r="H10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11">
+        <v>57</v>
+      </c>
+      <c r="D11">
+        <v>319</v>
+      </c>
+      <c r="F11">
+        <v>376</v>
+      </c>
+      <c r="G11" t="s">
+        <v>16</v>
+      </c>
+      <c r="H11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12">
+        <v>57</v>
+      </c>
+      <c r="D12">
+        <v>364</v>
+      </c>
+      <c r="F12">
+        <v>421</v>
+      </c>
+      <c r="G12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13">
+        <v>57</v>
+      </c>
+      <c r="D13">
+        <v>394</v>
+      </c>
+      <c r="F13">
+        <v>451</v>
+      </c>
+      <c r="G13" t="s">
+        <v>16</v>
+      </c>
+      <c r="H13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15">
+        <v>22</v>
+      </c>
+      <c r="D15">
+        <v>328</v>
+      </c>
+      <c r="E15">
+        <v>1001</v>
+      </c>
+      <c r="F15">
+        <v>1351</v>
+      </c>
+      <c r="G15" t="s">
+        <v>18</v>
+      </c>
+      <c r="H15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16">
+        <v>22</v>
+      </c>
+      <c r="D16">
+        <v>338</v>
+      </c>
+      <c r="E16">
+        <v>740</v>
+      </c>
+      <c r="F16">
+        <v>1100</v>
+      </c>
+      <c r="G16" t="s">
+        <v>18</v>
+      </c>
+      <c r="H16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17">
+        <v>22</v>
+      </c>
+      <c r="D17">
+        <v>347</v>
+      </c>
+      <c r="E17">
+        <v>1155</v>
+      </c>
+      <c r="F17">
+        <v>1524</v>
+      </c>
+      <c r="G17" t="s">
+        <v>18</v>
+      </c>
+      <c r="H17" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A9:H9"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>